<commit_message>
feat: 完整階段式分析流程 (Phase 1-4 + PhaseM)
- Phase 1 法人屬性：178,790 家公司，8 大基礎屬性
- PhaseM 聚類分析：206,797 家公司，7 種法人類型 (C0-C6)
- Phase 2 深度標籤：173,376 家公司，L1-L7 七層銷售情報（大檔案已排除）
- Phase 3 痛需熱圖：四路整合，生成熱圖與三輸出（推薦問項、開發卡、機會卡）
- Phase 4 v3 路徑分析：已在前一次提交完成

新增 .gitignore 規則：排除超過 50M 的大檔案（phase2_deep_labels.jsonl 等）
更新主要 notebook：L-Phase2深度標籤.ipynb, L-Phase3痛需熱圖.ipynb, 商機等級.ipynb
更新甘特圖：v4_7 → v4_8

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LLM系統開發甘特圖_v4_7.xlsx
+++ b/LLM系統開發甘特圖_v4_7.xlsx
@@ -1808,10 +1808,11 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="44" customWidth="1"/>
+    <col min="2" max="2" width="47.1428571428571" customWidth="1"/>
     <col min="3" max="3" width="12.1428571428571" customWidth="1"/>
     <col min="4" max="4" width="9.85714285714286" customWidth="1"/>
-    <col min="5" max="17" width="6" customWidth="1"/>
+    <col min="5" max="5" width="19.2857142857143" customWidth="1"/>
+    <col min="6" max="17" width="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:1">
@@ -2142,7 +2143,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1" spans="1:17">
+    <row r="9" ht="17" customHeight="1" spans="1:17">
       <c r="A9" s="20" t="s">
         <v>44</v>
       </c>
@@ -2619,7 +2620,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1" spans="1:17">
+    <row r="18" ht="24" customHeight="1" spans="1:17">
       <c r="A18" s="32" t="s">
         <v>62</v>
       </c>
@@ -2778,7 +2779,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1" spans="1:17">
+    <row r="21" spans="1:17">
       <c r="A21" s="37" t="s">
         <v>68</v>
       </c>
@@ -2990,7 +2991,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1" spans="1:17">
+    <row r="25" ht="17" customHeight="1" spans="1:17">
       <c r="A25" s="42" t="s">
         <v>77</v>
       </c>
@@ -3202,7 +3203,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1" spans="1:17">
+    <row r="29" ht="16" customHeight="1" spans="1:17">
       <c r="A29" s="46" t="s">
         <v>82</v>
       </c>
@@ -3255,7 +3256,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" ht="16" customHeight="1" spans="1:17">
+    <row r="30" spans="1:17">
       <c r="A30" s="12" t="s">
         <v>2</v>
       </c>

</xml_diff>